<commit_message>
chore: test workbooks follow the new sign-up flow; Arabic pass fixes
The plan and results now cover the role chooser, shop-owner documents and the
24-hour notice (67 checks). The onboarding screen is titled Create account and
the document size reads 1 KB in Arabic.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/Masari_Test_Plan.xlsx
+++ b/docs/demo/Masari_Test_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$F$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$F$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -761,17 +761,29 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Maps are grey or empty?</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>The maps load tiles from OpenStreetMap, so the emulator needs internet. If a map is a grey box, close the emulator and start it again with: emulator -avd Medium_Phone_API_36.0 -no-snapshot-load -dns-server 8.8.8.8,1.1.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>NOT IN SCOPE (do not report as bugs)</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Real SMS delivery (codes come from otp.txt), push notifications, payments, fares and earnings amounts, live tracking, PDF or Excel exports, maps and checkpoint feeds (switched off), and anything on a real server.</t>
         </is>
@@ -788,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1468,12 +1480,12 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Sign-in screen → "Create an invited account" → Passenger → enter the passenger invitation code and phone +970590002001 → Send verification code</t>
+          <t>Sign-in screen → "New to Masari? Create an account"</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>A code-entry screen appears with a resend countdown</t>
+          <t>A screen asks "How will you use Masari?" with three choices: Normal user, Driver, Shop owner. Normal user opens the email sign-up form; Driver and Shop owner open the invitation-code and phone screen with the role already chosen; Back returns to sign-in</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
@@ -1516,12 +1528,12 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Enter the right code (from otp.txt), then name, a password of at least 15 characters, tick the three consents, Create account</t>
+          <t>Choose Shop owner (invitation code and +970590002003), enter the right code (from otp.txt), then name, a password of at least 15 characters, tick the three consents, Create account</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Account created; the passenger can sign in and is active straight away</t>
+          <t>Account created; the screen says the account is pending and an admin review usually takes up to 24 hours</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
@@ -1540,7 +1552,7 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Repeat C01–C03 for the driver (+970590002002)</t>
+          <t>Repeat for the driver (+970590002002)</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
@@ -1756,12 +1768,12 @@
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Repeat C01–C03 for the merchant (+970590002003); Admin approves it (A09)</t>
+          <t>Admin approves the shop owner from C03 (A09), then sign in on the phone with their phone number and password</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Same pending → approved path; the merchant signs in</t>
+          <t>Same pending → approved path; the merchant home opens</t>
         </is>
       </c>
       <c r="E40" s="11" t="n"/>
@@ -1818,22 +1830,22 @@
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up with invitation</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Passenger: open the seeded request and its match</t>
+          <t>Shop owner (pending, from C03): Add a document → choose licence.jpg (type "Commercial register")</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>The request and a match result are shown</t>
+          <t>The pending screen shows "Verification documents" asking for the commercial register, national ID and shop photo; the file appears in the list as "Commercial register · 1 KB"</t>
         </is>
       </c>
       <c r="E43" s="11" t="n"/>
@@ -1842,22 +1854,22 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up with invitation</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>Merchant: open the seeded order</t>
+          <t>In the Admin site, Users → the pending shop owner → Approve (or Reject)</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>Five parcels and their batch are shown</t>
+          <t>The shop owner's documents are listed with a Download button before you decide; the downloaded file opens and is the right file</t>
         </is>
       </c>
       <c r="E44" s="11" t="n"/>
@@ -1866,7 +1878,7 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
@@ -1876,12 +1888,12 @@
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Admin: open the Matching page; if there is no match yet, run matching</t>
+          <t>Passenger: open the seeded request and its match</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>One combined passenger+parcel match exists, with a score breakdown</t>
+          <t>The request and a match result are shown</t>
         </is>
       </c>
       <c r="E45" s="11" t="n"/>
@@ -1890,7 +1902,7 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -1900,12 +1912,12 @@
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Driver (the selected one): open the inbox</t>
+          <t>Merchant: open the seeded order</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>The match is there; the other driver's inbox is empty</t>
+          <t>Five parcels and their batch are shown</t>
         </is>
       </c>
       <c r="E46" s="11" t="n"/>
@@ -1914,7 +1926,7 @@
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -1924,12 +1936,12 @@
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Driver: accept the match</t>
+          <t>Admin: open the Matching page; if there is no match yet, run matching</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>Exactly one trip is created</t>
+          <t>One combined passenger+parcel match exists, with a score breakdown</t>
         </is>
       </c>
       <c r="E47" s="11" t="n"/>
@@ -1938,7 +1950,7 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -1948,12 +1960,12 @@
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Driver: advance pickup → picked up → in transit (and simulate points)</t>
+          <t>Driver (the selected one): open the inbox</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>Only the next valid action is offered each time</t>
+          <t>The match is there; the other driver's inbox is empty</t>
         </is>
       </c>
       <c r="E48" s="11" t="n"/>
@@ -1962,7 +1974,7 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -1972,12 +1984,12 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Passenger and merchant: open their trip</t>
+          <t>Driver: accept the match</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Both see the same trip and the same latest location; read-only</t>
+          <t>Exactly one trip is created</t>
         </is>
       </c>
       <c r="E49" s="11" t="n"/>
@@ -1986,7 +1998,7 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -1996,12 +2008,12 @@
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>Passenger and merchant: bell and Notifications tab</t>
+          <t>Driver: advance pickup → picked up → in transit (and simulate points)</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>A "match accepted" and "trip update" entries; tapping one clears its dot; "Mark all as read" works</t>
+          <t>Only the next valid action is offered each time</t>
         </is>
       </c>
       <c r="E50" s="11" t="n"/>
@@ -2010,7 +2022,7 @@
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -2020,12 +2032,12 @@
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Driver: complete the trip</t>
+          <t>Passenger and merchant: open their trip</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Trip shows completed on all three phones and in the Admin</t>
+          <t>Both see the same trip and the same latest location; read-only</t>
         </is>
       </c>
       <c r="E51" s="11" t="n"/>
@@ -2034,7 +2046,7 @@
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
@@ -2044,12 +2056,12 @@
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Tracking wording</t>
+          <t>Passenger and merchant: bell and Notifications tab</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Anywhere location appears it is described as simulated, never as live GPS</t>
+          <t>A "match accepted" and "trip update" entries; tapping one clears its dot; "Mark all as read" works</t>
         </is>
       </c>
       <c r="E52" s="11" t="n"/>
@@ -2058,22 +2070,22 @@
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Main story (passenger, merchant, driver)</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>Driver: Earnings/performance tab</t>
+          <t>Driver: complete the trip</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Completed-trip counts shown; earnings says it is not tracked (no invented amount)</t>
+          <t>Trip shows completed on all three phones and in the Admin</t>
         </is>
       </c>
       <c r="E53" s="11" t="n"/>
@@ -2082,22 +2094,22 @@
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Main story (passenger, merchant, driver)</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Same tab, acceptance rate</t>
+          <t>Tracking wording</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Under 5 answered offers it says the rate appears after 5; after accepting/rejecting 5 offers it shows a percentage and "x of y"</t>
+          <t>Anywhere location appears it is described as simulated, never as live GPS</t>
         </is>
       </c>
       <c r="E54" s="11" t="n"/>
@@ -2106,7 +2118,7 @@
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
@@ -2116,12 +2128,12 @@
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>Driver: reject an offer and accept another (needs fresh offers: reset)</t>
+          <t>Driver: Earnings/performance tab</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>The numbers in E02 move accordingly</t>
+          <t>Completed-trip counts shown; earnings says it is not tracked (no invented amount)</t>
         </is>
       </c>
       <c r="E55" s="11" t="n"/>
@@ -2130,7 +2142,7 @@
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
@@ -2140,12 +2152,12 @@
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Merchant: Reports tab</t>
+          <t>Same tab, acceptance rate</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>Orders, parcels and deliveries by status; matches the Admin report for that merchant</t>
+          <t>Under 5 answered offers it says the rate appears after 5; after accepting/rejecting 5 offers it shows a percentage and "x of y"</t>
         </is>
       </c>
       <c r="E56" s="11" t="n"/>
@@ -2154,7 +2166,7 @@
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
@@ -2164,12 +2176,12 @@
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>Passenger on a trip: Report a problem → Delay → write a sentence → Send</t>
+          <t>Driver: reject an offer and accept another (needs fresh offers: reset)</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Confirmation; the sheet says it is not an emergency service</t>
+          <t>The numbers in E02 move accordingly</t>
         </is>
       </c>
       <c r="E57" s="11" t="n"/>
@@ -2178,7 +2190,7 @@
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
@@ -2188,12 +2200,12 @@
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Send 11 reports without any being resolved</t>
+          <t>Merchant: Reports tab</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>The 11th is refused with a message about too many open reports</t>
+          <t>Orders, parcels and deliveries by status; matches the Admin report for that merchant</t>
         </is>
       </c>
       <c r="E58" s="11" t="n"/>
@@ -2202,7 +2214,7 @@
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
@@ -2212,12 +2224,12 @@
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>Admin: Incidents</t>
+          <t>Passenger on a trip: Report a problem → Delay → write a sentence → Send</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>The report from E05 is there (see A16); after you resolve it, the passenger gets two new notifications and does not see your internal note</t>
+          <t>Confirmation; the sheet says it is not an emergency service</t>
         </is>
       </c>
       <c r="E59" s="11" t="n"/>
@@ -2226,7 +2238,7 @@
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
@@ -2236,12 +2248,12 @@
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Driver: go online/offline</t>
+          <t>Send 11 reports without any being resolved</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>The state changes once per tap and survives closing the app</t>
+          <t>The 11th is refused with a message about too many open reports</t>
         </is>
       </c>
       <c r="E60" s="11" t="n"/>
@@ -2250,22 +2262,22 @@
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>F01</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Smaller features</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Admin site: sign in as a passenger (using a passenger's email and password)</t>
+          <t>Admin: Incidents</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>The report from E05 is there (see A16); after you resolve it, the passenger gets two new notifications and does not see your internal note</t>
         </is>
       </c>
       <c r="E61" s="11" t="n"/>
@@ -2274,22 +2286,22 @@
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Smaller features</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>A pending merchant or driver signs in on the phone</t>
+          <t>Driver: go online/offline</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Refused with a clear message</t>
+          <t>The state changes once per tap and survives closing the app</t>
         </is>
       </c>
       <c r="E62" s="11" t="n"/>
@@ -2298,7 +2310,7 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
@@ -2308,7 +2320,7 @@
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>After the Admin rejects a driver with a reason, sign in as that driver</t>
+          <t>Admin site: sign in as a passenger (using a passenger's email and password)</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
@@ -2322,7 +2334,7 @@
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -2332,12 +2344,12 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>As a passenger, try to open driver or merchant screens (via the menu only; no URL tricks)</t>
+          <t>A pending merchant or driver signs in on the phone</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>Not reachable</t>
+          <t>Refused with a clear message</t>
         </is>
       </c>
       <c r="E64" s="11" t="n"/>
@@ -2346,7 +2358,7 @@
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
@@ -2356,12 +2368,12 @@
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>Admin downloads a driver document, then the applicant is approved: can the applicant still upload?</t>
+          <t>After the Admin rejects a driver with a reason, sign in as that driver</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>No: uploading is closed once a decision is made</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="E65" s="11" t="n"/>
@@ -2370,7 +2382,7 @@
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -2380,20 +2392,68 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>Look through every screen for the words "push notification", "emergency", "live GPS", "payment", "earnings" used as if they work</t>
+          <t>As a passenger, try to open driver or merchant screens (via the menu only; no URL tricks)</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>None claim a feature that is not built</t>
+          <t>Not reachable</t>
         </is>
       </c>
       <c r="E66" s="11" t="n"/>
       <c r="F66" s="11" t="n"/>
     </row>
+    <row r="67">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>Admin downloads a driver document, then the applicant is approved: can the applicant still upload?</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>No: uploading is closed once a decision is made</t>
+        </is>
+      </c>
+      <c r="E67" s="11" t="n"/>
+      <c r="F67" s="11" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C68" s="10" t="inlineStr">
+        <is>
+          <t>Look through every screen for the words "push notification", "emergency", "live GPS", "payment", "earnings" used as if they work</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr">
+        <is>
+          <t>None claim a feature that is not built</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="n"/>
+      <c r="F68" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F66"/>
-  <conditionalFormatting sqref="E2:E66">
+  <autoFilter ref="A1:F68"/>
+  <conditionalFormatting sqref="E2:E68">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2405,7 +2465,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose PASS, FAIL or SKIP." type="list">
+    <dataValidation sqref="E2:E68" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose PASS, FAIL or SKIP." type="list">
       <formula1>"PASS,FAIL,SKIP"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2469,19 +2529,19 @@
         </is>
       </c>
       <c r="B2" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$66,"A*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$68,"A*")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"A*",Tests!$E$2:$E$66,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"A*",Tests!$E$2:$E$68,"PASS")</f>
         <v/>
       </c>
       <c r="D2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"A*",Tests!$E$2:$E$66,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"A*",Tests!$E$2:$E$68,"FAIL")</f>
         <v/>
       </c>
       <c r="E2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"A*",Tests!$E$2:$E$66,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"A*",Tests!$E$2:$E$68,"SKIP")</f>
         <v/>
       </c>
       <c r="F2" s="13">
@@ -2496,19 +2556,19 @@
         </is>
       </c>
       <c r="B3" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$66,"B*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$68,"B*")</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"B*",Tests!$E$2:$E$66,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"B*",Tests!$E$2:$E$68,"PASS")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"B*",Tests!$E$2:$E$66,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"B*",Tests!$E$2:$E$68,"FAIL")</f>
         <v/>
       </c>
       <c r="E3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"B*",Tests!$E$2:$E$66,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"B*",Tests!$E$2:$E$68,"SKIP")</f>
         <v/>
       </c>
       <c r="F3" s="13">
@@ -2523,19 +2583,19 @@
         </is>
       </c>
       <c r="B4" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$66,"C*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$68,"C*")</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"C*",Tests!$E$2:$E$66,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"C*",Tests!$E$2:$E$68,"PASS")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"C*",Tests!$E$2:$E$66,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"C*",Tests!$E$2:$E$68,"FAIL")</f>
         <v/>
       </c>
       <c r="E4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"C*",Tests!$E$2:$E$66,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"C*",Tests!$E$2:$E$68,"SKIP")</f>
         <v/>
       </c>
       <c r="F4" s="13">
@@ -2550,19 +2610,19 @@
         </is>
       </c>
       <c r="B5" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$66,"D*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$68,"D*")</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"D*",Tests!$E$2:$E$66,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"D*",Tests!$E$2:$E$68,"PASS")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"D*",Tests!$E$2:$E$66,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"D*",Tests!$E$2:$E$68,"FAIL")</f>
         <v/>
       </c>
       <c r="E5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"D*",Tests!$E$2:$E$66,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"D*",Tests!$E$2:$E$68,"SKIP")</f>
         <v/>
       </c>
       <c r="F5" s="13">
@@ -2577,19 +2637,19 @@
         </is>
       </c>
       <c r="B6" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$66,"E*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$68,"E*")</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"E*",Tests!$E$2:$E$66,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"E*",Tests!$E$2:$E$68,"PASS")</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"E*",Tests!$E$2:$E$66,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"E*",Tests!$E$2:$E$68,"FAIL")</f>
         <v/>
       </c>
       <c r="E6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"E*",Tests!$E$2:$E$66,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"E*",Tests!$E$2:$E$68,"SKIP")</f>
         <v/>
       </c>
       <c r="F6" s="13">
@@ -2604,19 +2664,19 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$66,"F*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$68,"F*")</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"F*",Tests!$E$2:$E$66,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"F*",Tests!$E$2:$E$68,"PASS")</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"F*",Tests!$E$2:$E$66,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"F*",Tests!$E$2:$E$68,"FAIL")</f>
         <v/>
       </c>
       <c r="E7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$66,"F*",Tests!$E$2:$E$66,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$68,"F*",Tests!$E$2:$E$68,"SKIP")</f>
         <v/>
       </c>
       <c r="F7" s="13">

</xml_diff>

<commit_message>
test-env: demo writes email and phone codes to files so a normal user can finish sign-up
Adds the normal-user path (C18) to the test plan and results.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/Masari_Test_Plan.xlsx
+++ b/docs/demo/Masari_Test_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$F$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$F$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -800,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1878,22 +1878,22 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up with invitation</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Passenger: open the seeded request and its match</t>
+          <t>Create account → Normal user → name, an email ending in @example.com, a password of at least 12 characters → Sign up; paste the token from email-codes.txt, tick the three documents, Continue; then enter a phone such as +970590003020, Send code, type the code from otp.txt, Continue</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>The request and a match result are shown</t>
+          <t>The passenger home opens; no invitation code and no admin approval were needed</t>
         </is>
       </c>
       <c r="E45" s="11" t="n"/>
@@ -1902,7 +1902,7 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -1912,12 +1912,12 @@
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Merchant: open the seeded order</t>
+          <t>Passenger: open the seeded request and its match</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>Five parcels and their batch are shown</t>
+          <t>The request and a match result are shown</t>
         </is>
       </c>
       <c r="E46" s="11" t="n"/>
@@ -1926,7 +1926,7 @@
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>D02</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
@@ -1936,12 +1936,12 @@
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Admin: open the Matching page; if there is no match yet, run matching</t>
+          <t>Merchant: open the seeded order</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>One combined passenger+parcel match exists, with a score breakdown</t>
+          <t>Five parcels and their batch are shown</t>
         </is>
       </c>
       <c r="E47" s="11" t="n"/>
@@ -1950,7 +1950,7 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>D03</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -1960,12 +1960,12 @@
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Driver (the selected one): open the inbox</t>
+          <t>Admin: open the Matching page; if there is no match yet, run matching</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>The match is there; the other driver's inbox is empty</t>
+          <t>One combined passenger+parcel match exists, with a score breakdown</t>
         </is>
       </c>
       <c r="E48" s="11" t="n"/>
@@ -1974,7 +1974,7 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>D04</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
@@ -1984,12 +1984,12 @@
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Driver: accept the match</t>
+          <t>Driver (the selected one): open the inbox</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Exactly one trip is created</t>
+          <t>The match is there; the other driver's inbox is empty</t>
         </is>
       </c>
       <c r="E49" s="11" t="n"/>
@@ -1998,7 +1998,7 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>D05</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
@@ -2008,12 +2008,12 @@
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>Driver: advance pickup → picked up → in transit (and simulate points)</t>
+          <t>Driver: accept the match</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>Only the next valid action is offered each time</t>
+          <t>Exactly one trip is created</t>
         </is>
       </c>
       <c r="E50" s="11" t="n"/>
@@ -2022,7 +2022,7 @@
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>D06</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Passenger and merchant: open their trip</t>
+          <t>Driver: advance pickup → picked up → in transit (and simulate points)</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Both see the same trip and the same latest location; read-only</t>
+          <t>Only the next valid action is offered each time</t>
         </is>
       </c>
       <c r="E51" s="11" t="n"/>
@@ -2046,7 +2046,7 @@
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>D07</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
@@ -2056,12 +2056,12 @@
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Passenger and merchant: bell and Notifications tab</t>
+          <t>Passenger and merchant: open their trip</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>A "match accepted" and "trip update" entries; tapping one clears its dot; "Mark all as read" works</t>
+          <t>Both see the same trip and the same latest location; read-only</t>
         </is>
       </c>
       <c r="E52" s="11" t="n"/>
@@ -2070,7 +2070,7 @@
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>D08</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>Driver: complete the trip</t>
+          <t>Passenger and merchant: bell and Notifications tab</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Trip shows completed on all three phones and in the Admin</t>
+          <t>A "match accepted" and "trip update" entries; tapping one clears its dot; "Mark all as read" works</t>
         </is>
       </c>
       <c r="E53" s="11" t="n"/>
@@ -2094,7 +2094,7 @@
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D09</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
@@ -2104,12 +2104,12 @@
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Tracking wording</t>
+          <t>Driver: complete the trip</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Anywhere location appears it is described as simulated, never as live GPS</t>
+          <t>Trip shows completed on all three phones and in the Admin</t>
         </is>
       </c>
       <c r="E54" s="11" t="n"/>
@@ -2118,22 +2118,22 @@
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Main story (passenger, merchant, driver)</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>Driver: Earnings/performance tab</t>
+          <t>Tracking wording</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>Completed-trip counts shown; earnings says it is not tracked (no invented amount)</t>
+          <t>Anywhere location appears it is described as simulated, never as live GPS</t>
         </is>
       </c>
       <c r="E55" s="11" t="n"/>
@@ -2142,7 +2142,7 @@
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>E01</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
@@ -2152,12 +2152,12 @@
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Same tab, acceptance rate</t>
+          <t>Driver: Earnings/performance tab</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>Under 5 answered offers it says the rate appears after 5; after accepting/rejecting 5 offers it shows a percentage and "x of y"</t>
+          <t>Completed-trip counts shown; earnings says it is not tracked (no invented amount)</t>
         </is>
       </c>
       <c r="E56" s="11" t="n"/>
@@ -2166,7 +2166,7 @@
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>E02</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>Driver: reject an offer and accept another (needs fresh offers: reset)</t>
+          <t>Same tab, acceptance rate</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>The numbers in E02 move accordingly</t>
+          <t>Under 5 answered offers it says the rate appears after 5; after accepting/rejecting 5 offers it shows a percentage and "x of y"</t>
         </is>
       </c>
       <c r="E57" s="11" t="n"/>
@@ -2190,7 +2190,7 @@
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>E03</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
@@ -2200,12 +2200,12 @@
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Merchant: Reports tab</t>
+          <t>Driver: reject an offer and accept another (needs fresh offers: reset)</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>Orders, parcels and deliveries by status; matches the Admin report for that merchant</t>
+          <t>The numbers in E02 move accordingly</t>
         </is>
       </c>
       <c r="E58" s="11" t="n"/>
@@ -2214,7 +2214,7 @@
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>E04</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
@@ -2224,12 +2224,12 @@
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>Passenger on a trip: Report a problem → Delay → write a sentence → Send</t>
+          <t>Merchant: Reports tab</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Confirmation; the sheet says it is not an emergency service</t>
+          <t>Orders, parcels and deliveries by status; matches the Admin report for that merchant</t>
         </is>
       </c>
       <c r="E59" s="11" t="n"/>
@@ -2238,7 +2238,7 @@
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>E05</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
@@ -2248,12 +2248,12 @@
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Send 11 reports without any being resolved</t>
+          <t>Passenger on a trip: Report a problem → Delay → write a sentence → Send</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>The 11th is refused with a message about too many open reports</t>
+          <t>Confirmation; the sheet says it is not an emergency service</t>
         </is>
       </c>
       <c r="E60" s="11" t="n"/>
@@ -2262,7 +2262,7 @@
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>E06</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
@@ -2272,12 +2272,12 @@
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Admin: Incidents</t>
+          <t>Send 11 reports without any being resolved</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>The report from E05 is there (see A16); after you resolve it, the passenger gets two new notifications and does not see your internal note</t>
+          <t>The 11th is refused with a message about too many open reports</t>
         </is>
       </c>
       <c r="E61" s="11" t="n"/>
@@ -2286,7 +2286,7 @@
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>E07</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -2296,12 +2296,12 @@
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Driver: go online/offline</t>
+          <t>Admin: Incidents</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>The state changes once per tap and survives closing the app</t>
+          <t>The report from E05 is there (see A16); after you resolve it, the passenger gets two new notifications and does not see your internal note</t>
         </is>
       </c>
       <c r="E62" s="11" t="n"/>
@@ -2310,22 +2310,22 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>F01</t>
+          <t>E08</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Smaller features</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Admin site: sign in as a passenger (using a passenger's email and password)</t>
+          <t>Driver: go online/offline</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>The state changes once per tap and survives closing the app</t>
         </is>
       </c>
       <c r="E63" s="11" t="n"/>
@@ -2334,7 +2334,7 @@
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>F01</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -2344,12 +2344,12 @@
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>A pending merchant or driver signs in on the phone</t>
+          <t>Admin site: sign in as a passenger (using a passenger's email and password)</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>Refused with a clear message</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="E64" s="11" t="n"/>
@@ -2358,7 +2358,7 @@
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>F02</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
@@ -2368,12 +2368,12 @@
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>After the Admin rejects a driver with a reason, sign in as that driver</t>
+          <t>A pending merchant or driver signs in on the phone</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>Refused with a clear message</t>
         </is>
       </c>
       <c r="E65" s="11" t="n"/>
@@ -2382,7 +2382,7 @@
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>F03</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -2392,12 +2392,12 @@
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>As a passenger, try to open driver or merchant screens (via the menu only; no URL tricks)</t>
+          <t>After the Admin rejects a driver with a reason, sign in as that driver</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>Not reachable</t>
+          <t>Refused</t>
         </is>
       </c>
       <c r="E66" s="11" t="n"/>
@@ -2406,7 +2406,7 @@
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>F04</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
@@ -2416,12 +2416,12 @@
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Admin downloads a driver document, then the applicant is approved: can the applicant still upload?</t>
+          <t>As a passenger, try to open driver or merchant screens (via the menu only; no URL tricks)</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>No: uploading is closed once a decision is made</t>
+          <t>Not reachable</t>
         </is>
       </c>
       <c r="E67" s="11" t="n"/>
@@ -2430,7 +2430,7 @@
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>F05</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -2440,20 +2440,44 @@
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Look through every screen for the words "push notification", "emergency", "live GPS", "payment", "earnings" used as if they work</t>
+          <t>Admin downloads a driver document, then the applicant is approved: can the applicant still upload?</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>None claim a feature that is not built</t>
+          <t>No: uploading is closed once a decision is made</t>
         </is>
       </c>
       <c r="E68" s="11" t="n"/>
       <c r="F68" s="11" t="n"/>
     </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C69" s="10" t="inlineStr">
+        <is>
+          <t>Look through every screen for the words "push notification", "emergency", "live GPS", "payment", "earnings" used as if they work</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>None claim a feature that is not built</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="n"/>
+      <c r="F69" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F68"/>
-  <conditionalFormatting sqref="E2:E68">
+  <autoFilter ref="A1:F69"/>
+  <conditionalFormatting sqref="E2:E69">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2465,7 +2489,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E68" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose PASS, FAIL or SKIP." type="list">
+    <dataValidation sqref="E2:E69" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose PASS, FAIL or SKIP." type="list">
       <formula1>"PASS,FAIL,SKIP"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2529,19 +2553,19 @@
         </is>
       </c>
       <c r="B2" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$68,"A*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$69,"A*")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"A*",Tests!$E$2:$E$68,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"A*",Tests!$E$2:$E$69,"PASS")</f>
         <v/>
       </c>
       <c r="D2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"A*",Tests!$E$2:$E$68,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"A*",Tests!$E$2:$E$69,"FAIL")</f>
         <v/>
       </c>
       <c r="E2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"A*",Tests!$E$2:$E$68,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"A*",Tests!$E$2:$E$69,"SKIP")</f>
         <v/>
       </c>
       <c r="F2" s="13">
@@ -2556,19 +2580,19 @@
         </is>
       </c>
       <c r="B3" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$68,"B*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$69,"B*")</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"B*",Tests!$E$2:$E$68,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"B*",Tests!$E$2:$E$69,"PASS")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"B*",Tests!$E$2:$E$68,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"B*",Tests!$E$2:$E$69,"FAIL")</f>
         <v/>
       </c>
       <c r="E3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"B*",Tests!$E$2:$E$68,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"B*",Tests!$E$2:$E$69,"SKIP")</f>
         <v/>
       </c>
       <c r="F3" s="13">
@@ -2583,19 +2607,19 @@
         </is>
       </c>
       <c r="B4" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$68,"C*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$69,"C*")</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"C*",Tests!$E$2:$E$68,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"C*",Tests!$E$2:$E$69,"PASS")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"C*",Tests!$E$2:$E$68,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"C*",Tests!$E$2:$E$69,"FAIL")</f>
         <v/>
       </c>
       <c r="E4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"C*",Tests!$E$2:$E$68,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"C*",Tests!$E$2:$E$69,"SKIP")</f>
         <v/>
       </c>
       <c r="F4" s="13">
@@ -2610,19 +2634,19 @@
         </is>
       </c>
       <c r="B5" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$68,"D*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$69,"D*")</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"D*",Tests!$E$2:$E$68,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"D*",Tests!$E$2:$E$69,"PASS")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"D*",Tests!$E$2:$E$68,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"D*",Tests!$E$2:$E$69,"FAIL")</f>
         <v/>
       </c>
       <c r="E5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"D*",Tests!$E$2:$E$68,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"D*",Tests!$E$2:$E$69,"SKIP")</f>
         <v/>
       </c>
       <c r="F5" s="13">
@@ -2637,19 +2661,19 @@
         </is>
       </c>
       <c r="B6" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$68,"E*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$69,"E*")</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"E*",Tests!$E$2:$E$68,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"E*",Tests!$E$2:$E$69,"PASS")</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"E*",Tests!$E$2:$E$68,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"E*",Tests!$E$2:$E$69,"FAIL")</f>
         <v/>
       </c>
       <c r="E6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"E*",Tests!$E$2:$E$68,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"E*",Tests!$E$2:$E$69,"SKIP")</f>
         <v/>
       </c>
       <c r="F6" s="13">
@@ -2664,19 +2688,19 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$68,"F*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$69,"F*")</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"F*",Tests!$E$2:$E$68,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"F*",Tests!$E$2:$E$69,"PASS")</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"F*",Tests!$E$2:$E$68,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"F*",Tests!$E$2:$E$69,"FAIL")</f>
         <v/>
       </c>
       <c r="E7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$68,"F*",Tests!$E$2:$E$68,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$69,"F*",Tests!$E$2:$E$69,"SKIP")</f>
         <v/>
       </c>
       <c r="F7" s="13">

</xml_diff>

<commit_message>
test-env: demo checks cover the new features (email codes, open sign-up, fares, parcels, handover, trust, AI, expiry, bulk, metrics)
Adds scripts/test-env/new-feature-checks.mjs (41 API checks, run by run-checks.mjs, shared helpers in check-kit.mjs), turns on the route switches for the local test environment only, marks the automated check phone numbers as demo data, and adds the matching rows to TEST_PLAN.md and the two workbooks.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/Masari_Test_Plan.xlsx
+++ b/docs/demo/Masari_Test_Plan.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$F$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$1:$F$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,11 +130,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -170,6 +171,36 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00E7E6E6"/>
+          <bgColor rgb="00E7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor rgb="00E7E6E6"/>
         </patternFill>
       </fill>
@@ -557,6 +588,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -601,6 +633,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -633,6 +666,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -697,7 +731,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>No real SMS is sent. Open .staging-data/test-env/otp.txt and use the newest line.</t>
+          <t>No real SMS is sent. Open .staging-data/test-env/otp.txt and use the newest line.  Email sign-up and password-reset codes: the newest line for that email in .staging-data/test-env/email-codes.txt.</t>
         </is>
       </c>
     </row>
@@ -773,6 +807,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -785,7 +820,7 @@
       <c r="A27" s="5" t="inlineStr"/>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Real SMS delivery (codes come from otp.txt), push notifications, payments, fares and earnings amounts, live tracking, PDF or Excel exports, maps and checkpoint feeds (switched off), and anything on a real server.</t>
+          <t>Real SMS delivery (codes come from otp.txt), push notifications, payments and real money movement (route fares are display-only estimates; earnings amounts are not tracked), live tracking, PDF or Excel exports, maps and checkpoint feeds (switched off), and anything on a real server.</t>
         </is>
       </c>
     </row>
@@ -800,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1302,22 +1337,22 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>A20</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Phone: signing in</t>
+          <t>Admin site</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Open the app</t>
+          <t>Reports page → Success metrics (or GET /api/v1/admin/success-metrics, and /export for the CSV): open it as the Admin, then try it as a passenger and without signing in</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Sign-in screen, Arabic by default, right-to-left</t>
+          <t>Admin: figures for the last 30 days with the previous period for comparison, a CSV download; passenger: refused (403); not signed in: 401; a start date after the end date, or a range over a year, is refused</t>
         </is>
       </c>
       <c r="E21" s="11" t="n"/>
@@ -1326,22 +1361,22 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>A21</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Phone: signing in</t>
+          <t>Admin site</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Switch to English with the globe icon</t>
+          <t>Matching / Batching page → Simulated comparison tab (or GET /api/v1/compare/simulation?seed=7)</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Everything flips to English, left-to-right; switch back works</t>
+          <t>Manual, nearest-driver and Masari results, labelled as simulated; the same seed always gives the same numbers, another seed differs; nothing is written; passengers cannot call it</t>
         </is>
       </c>
       <c r="E22" s="11" t="n"/>
@@ -1350,7 +1385,7 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
@@ -1360,12 +1395,12 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Wrong email/password</t>
+          <t>Open the app</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>A clear "incorrect" message, not a crash or a network error</t>
+          <t>Sign-in screen, Arabic by default, right-to-left</t>
         </is>
       </c>
       <c r="E23" s="11" t="n"/>
@@ -1374,7 +1409,7 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -1384,12 +1419,12 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Sign in as the demo passenger</t>
+          <t>Switch to English with the globe icon</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Passenger home opens</t>
+          <t>Everything flips to English, left-to-right; switch back works</t>
         </is>
       </c>
       <c r="E24" s="11" t="n"/>
@@ -1398,7 +1433,7 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -1408,12 +1443,12 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Sign out, sign in as the demo driver, then the demo merchant</t>
+          <t>Wrong email/password</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Each role sees its own home and tabs, and none of the other roles' screens</t>
+          <t>A clear "incorrect" message, not a crash or a network error</t>
         </is>
       </c>
       <c r="E25" s="11" t="n"/>
@@ -1422,7 +1457,7 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>B06</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -1432,12 +1467,12 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Close the app completely and reopen it</t>
+          <t>Sign in as the demo passenger</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>You are still signed in (or sent to sign-in, but never to a broken screen)</t>
+          <t>Passenger home opens</t>
         </is>
       </c>
       <c r="E26" s="11" t="n"/>
@@ -1446,7 +1481,7 @@
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>B07</t>
+          <t>B05</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -1456,12 +1491,12 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Turn the emulator's internet off (airplane mode) and open a list</t>
+          <t>Sign out, sign in as the demo driver, then the demo merchant</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>A friendly offline/error message with a retry; no crash</t>
+          <t>Each role sees its own home and tabs, and none of the other roles' screens</t>
         </is>
       </c>
       <c r="E27" s="11" t="n"/>
@@ -1470,22 +1505,22 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>C01</t>
+          <t>B06</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: signing in</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Sign-in screen → "New to Masari? Create an account"</t>
+          <t>Close the app completely and reopen it</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>A screen asks "How will you use Masari?" with three choices: Normal user, Driver, Shop owner. Normal user opens the email sign-up form; Driver and Shop owner open the invitation-code and phone screen with the role already chosen; Back returns to sign-in</t>
+          <t>You are still signed in (or sent to sign-in, but never to a broken screen)</t>
         </is>
       </c>
       <c r="E28" s="11" t="n"/>
@@ -1494,22 +1529,22 @@
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>C02</t>
+          <t>B07</t>
         </is>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: signing in</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Enter a wrong code</t>
+          <t>Turn the emulator's internet off (airplane mode) and open a list</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>A clear error; you can try again</t>
+          <t>A friendly offline/error message with a retry; no crash</t>
         </is>
       </c>
       <c r="E29" s="11" t="n"/>
@@ -1518,22 +1553,22 @@
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>C03</t>
+          <t>C01</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Choose Shop owner (invitation code and +970590002003), enter the right code (from otp.txt), then name, a password of at least 15 characters, tick the three consents, Create account</t>
+          <t>Sign-in screen → "New to Masari? Create an account"</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Account created; the screen says the account is pending and an admin review usually takes up to 24 hours</t>
+          <t>A screen asks "How will you use Masari?" with three choices: Normal user, Driver, Shop owner. Normal user opens the email sign-up form; Driver and Shop owner open the invitation-code and phone screen with the role already chosen; Back returns to sign-in</t>
         </is>
       </c>
       <c r="E30" s="11" t="n"/>
@@ -1542,22 +1577,22 @@
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>C04</t>
+          <t>C02</t>
         </is>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Repeat for the driver (+970590002002)</t>
+          <t>Enter a wrong code</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>The screen says "Application under review" and shows a "Verification documents" card</t>
+          <t>A clear error; you can try again</t>
         </is>
       </c>
       <c r="E31" s="11" t="n"/>
@@ -1566,22 +1601,22 @@
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>C05</t>
+          <t>C03</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Driver: Add a document → choose licence.jpg (type "Driving licence")</t>
+          <t>Choose Shop owner (invitation code and +970590002003), enter the right code (from otp.txt), then name, a password of at least 15 characters, tick the three consents, Create account</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>It appears in the list as "Driving licence · 1 KB"</t>
+          <t>Account created; the screen says the account is pending and an admin review usually takes up to 24 hours</t>
         </is>
       </c>
       <c r="E32" s="11" t="n"/>
@@ -1590,22 +1625,22 @@
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>C06</t>
+          <t>C04</t>
         </is>
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Add vehicle-registration.pdf with type "Vehicle registration"</t>
+          <t>Repeat for the driver (+970590002002)</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>It appears in the list</t>
+          <t>The screen says "Application under review" and shows a "Verification documents" card</t>
         </is>
       </c>
       <c r="E33" s="11" t="n"/>
@@ -1614,22 +1649,22 @@
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>C07</t>
+          <t>C05</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Add not-really-an-image.jpg</t>
+          <t>Driver: Add a document → choose licence.jpg (type "Driving licence")</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>Refused with "Only JPEG, PNG or PDF files can be uploaded"; nothing added</t>
+          <t>It appears in the list as "Driving licence · 1 KB"</t>
         </is>
       </c>
       <c r="E34" s="11" t="n"/>
@@ -1638,22 +1673,22 @@
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>C08</t>
+          <t>C06</t>
         </is>
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Tap the bin on one document</t>
+          <t>Add vehicle-registration.pdf with type "Vehicle registration"</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>It disappears from the list</t>
+          <t>It appears in the list</t>
         </is>
       </c>
       <c r="E35" s="11" t="n"/>
@@ -1662,22 +1697,22 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>C09</t>
+          <t>C07</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Try to add more than 6 documents</t>
+          <t>Add not-really-an-image.jpg</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>After 6 the Add button is disabled or a limit message shows</t>
+          <t>Refused with "Only JPEG, PNG or PDF files can be uploaded"; nothing added</t>
         </is>
       </c>
       <c r="E36" s="11" t="n"/>
@@ -1686,22 +1721,22 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>C10</t>
+          <t>C08</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>In the Admin site, open that driver's review</t>
+          <t>Tap the bin on one document</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>The uploaded documents are listed with a Download button; the downloaded file opens and is the right file</t>
+          <t>It disappears from the list</t>
         </is>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -1710,22 +1745,22 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>C11</t>
+          <t>C09</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Try to sign in on the phone as the new (pending) driver</t>
+          <t>Try to add more than 6 documents</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>You are not let in (account pending), with a clear message</t>
+          <t>After 6 the Add button is disabled or a limit message shows</t>
         </is>
       </c>
       <c r="E38" s="11" t="n"/>
@@ -1734,22 +1769,22 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>C12</t>
+          <t>C10</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Admin approves that driver (A13), then press Refresh in the app's pending screen</t>
+          <t>In the Admin site, open that driver's review</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>It now says approved and offers sign-in; sign-in works</t>
+          <t>The uploaded documents are listed with a Download button; the downloaded file opens and is the right file</t>
         </is>
       </c>
       <c r="E39" s="11" t="n"/>
@@ -1758,22 +1793,22 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>C13</t>
+          <t>C11</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
-          <t>Admin approves the shop owner from C03 (A09), then sign in on the phone with their phone number and password</t>
+          <t>Try to sign in on the phone as the new (pending) driver</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Same pending → approved path; the merchant home opens</t>
+          <t>You are not let in (account pending), with a clear message</t>
         </is>
       </c>
       <c r="E40" s="11" t="n"/>
@@ -1782,22 +1817,22 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>C14</t>
+          <t>C12</t>
         </is>
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Use an invitation code twice, or a code with the wrong phone</t>
+          <t>Admin approves that driver (A13), then press Refresh in the app's pending screen</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Refused without revealing why</t>
+          <t>It now says approved and offers sign-in; sign-in works</t>
         </is>
       </c>
       <c r="E41" s="11" t="n"/>
@@ -1806,22 +1841,22 @@
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>C15</t>
+          <t>C13</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
-          <t>Sign-in screen → "Check an existing application" with a pending applicant's phone and password</t>
+          <t>Admin approves the shop owner from C03 (A09), then sign in on the phone with their phone number and password</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Shows the application status</t>
+          <t>Same pending → approved path; the merchant home opens</t>
         </is>
       </c>
       <c r="E42" s="11" t="n"/>
@@ -1830,22 +1865,22 @@
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C14</t>
         </is>
       </c>
       <c r="B43" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Shop owner (pending, from C03): Add a document → choose licence.jpg (type "Commercial register")</t>
+          <t>Use an invitation code twice, or a code with the wrong phone</t>
         </is>
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>The pending screen shows "Verification documents" asking for the commercial register, national ID and shop photo; the file appears in the list as "Commercial register · 1 KB"</t>
+          <t>Refused without revealing why</t>
         </is>
       </c>
       <c r="E43" s="11" t="n"/>
@@ -1854,22 +1889,22 @@
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>C17</t>
+          <t>C15</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>In the Admin site, Users → the pending shop owner → Approve (or Reject)</t>
+          <t>Sign-in screen → "Check an existing application" with a pending applicant's phone and password</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>The shop owner's documents are listed with a Download button before you decide; the downloaded file opens and is the right file</t>
+          <t>Shows the application status</t>
         </is>
       </c>
       <c r="E44" s="11" t="n"/>
@@ -1878,22 +1913,22 @@
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>C18</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Create account → Normal user → name, an email ending in @example.com, a password of at least 12 characters → Sign up; type the six-digit code from email-codes.txt, tick the three documents, Continue; then enter a phone such as +970590003020, Send code, type the code from otp.txt, Continue</t>
+          <t>Shop owner (pending, from C03): Add a document → choose licence.jpg (type "Commercial register")</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>The passenger home opens; no invitation code and no admin approval were needed</t>
+          <t>The pending screen shows "Verification documents" asking for the commercial register, national ID and shop photo; the file appears in the list as "Commercial register · 1 KB"</t>
         </is>
       </c>
       <c r="E45" s="11" t="n"/>
@@ -1902,22 +1937,22 @@
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>D01</t>
+          <t>C17</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
-          <t>Passenger: open the seeded request and its match</t>
+          <t>In the Admin site, Users → the pending shop owner → Approve (or Reject)</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>The request and a match result are shown</t>
+          <t>The shop owner's documents are listed with a Download button before you decide; the downloaded file opens and is the right file</t>
         </is>
       </c>
       <c r="E46" s="11" t="n"/>
@@ -1926,22 +1961,22 @@
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>D02</t>
+          <t>C18</t>
         </is>
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Merchant: open the seeded order</t>
+          <t>Create account → Normal user → name, an email ending in @example.com, a password of at least 12 characters → Sign up; type the six-digit code from email-codes.txt, tick the three documents, Continue; then enter a phone such as +970590003020, Send code, type the code from otp.txt, Continue</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>Five parcels and their batch are shown</t>
+          <t>The passenger home opens; no invitation code and no admin approval were needed</t>
         </is>
       </c>
       <c r="E47" s="11" t="n"/>
@@ -1950,22 +1985,22 @@
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>D03</t>
+          <t>C19</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Admin: open the Matching page; if there is no match yet, run matching</t>
+          <t>Open registration (the local test environment turns it on). Create account → Driver. Leave the invitation code empty (it says "Invitation code (optional)"), enter a new phone such as +970590004001, Send code, type the code from otp.txt</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>One combined passenger+parcel match exists, with a score breakdown</t>
+          <t>The code screen opens without any invitation code</t>
         </is>
       </c>
       <c r="E48" s="11" t="n"/>
@@ -1974,22 +2009,22 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>D04</t>
+          <t>C20</t>
         </is>
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Driver (the selected one): open the inbox</t>
+          <t>Enter a wrong code, then the right one; then name, a password of at least 15 characters, tick the three consents, Create account</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>The match is there; the other driver's inbox is empty</t>
+          <t>Account created; the screen says "Upload your documents" (not "Application under review"); the button "Send for review" is disabled and lists what is still needed</t>
         </is>
       </c>
       <c r="E49" s="11" t="n"/>
@@ -1998,22 +2033,22 @@
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>D05</t>
+          <t>C21</t>
         </is>
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>Driver: accept the match</t>
+          <t>Add licence.jpg (Driving licence) and vehicle-registration.pdf (Vehicle registration) only</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>Exactly one trip is created</t>
+          <t>"Send for review" stays disabled; "Still needed" names the national ID</t>
         </is>
       </c>
       <c r="E50" s="11" t="n"/>
@@ -2022,22 +2057,22 @@
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>D06</t>
+          <t>C22</t>
         </is>
       </c>
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Driver: advance pickup → picked up → in transit (and simulate points)</t>
+          <t>In the Admin site, look in Users and the driver approvals queue for that driver</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Only the next valid action is offered each time</t>
+          <t>The driver is not in the review queue yet; approving or rejecting is refused (not submitted)</t>
         </is>
       </c>
       <c r="E51" s="11" t="n"/>
@@ -2046,22 +2081,22 @@
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>D07</t>
+          <t>C23</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Passenger and merchant: open their trip</t>
+          <t>Add a National ID document, then press "Send for review"</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Both see the same trip and the same latest location; read-only</t>
+          <t>The screen changes to "Application under review" and says review usually takes up to 24 hours</t>
         </is>
       </c>
       <c r="E52" s="11" t="n"/>
@@ -2070,22 +2105,22 @@
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>D08</t>
+          <t>C24</t>
         </is>
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>Passenger and merchant: bell and Notifications tab</t>
+          <t>In the Admin site open the driver approvals queue</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>A "match accepted" and "trip update" entries; tapping one clears its dot; "Mark all as read" works</t>
+          <t>The driver is listed; the three documents have Download buttons and open correctly; Approve works; the phone then signs in</t>
         </is>
       </c>
       <c r="E53" s="11" t="n"/>
@@ -2094,22 +2129,22 @@
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>D09</t>
+          <t>C25</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Driver: complete the trip</t>
+          <t>Create account → Shop owner with no invitation code (+970590004002); upload commercial register and national ID only</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>Trip shows completed on all three phones and in the Admin</t>
+          <t>"Send for review" stays disabled until the shop photo is added; then it submits and the shop owner appears in Users as a pending merchant that can be approved</t>
         </is>
       </c>
       <c r="E54" s="11" t="n"/>
@@ -2118,22 +2153,22 @@
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>C26</t>
         </is>
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>Main story (passenger, merchant, driver)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>Tracking wording</t>
+          <t>Open registration, start with a phone number that already has an account, type the code from otp.txt, then fill the form</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>Anywhere location appears it is described as simulated, never as live GPS</t>
+          <t>The first screens look exactly like a new number; only at Create account does it say the registration could not be completed</t>
         </is>
       </c>
       <c r="E55" s="11" t="n"/>
@@ -2142,22 +2177,22 @@
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>E01</t>
+          <t>C27</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Driver: Earnings/performance tab</t>
+          <t>Start sign-up again with the same phone number twice, then use the first code</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>Completed-trip counts shown; earnings says it is not tracked (no invented amount)</t>
+          <t>The older attempt no longer works; only the newest code and screen continue</t>
         </is>
       </c>
       <c r="E56" s="11" t="n"/>
@@ -2166,22 +2201,22 @@
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>E02</t>
+          <t>C28</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>Same tab, acceptance rate</t>
+          <t>Request a code for the same phone more than 5 times in a day, or start more than 10 sign-ups from the one phone in an hour</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Under 5 answered offers it says the rate appears after 5; after accepting/rejecting 5 offers it shows a percentage and "x of y"</t>
+          <t>The app shows a "too many attempts" message; no further codes are produced in otp.txt</t>
         </is>
       </c>
       <c r="E57" s="11" t="n"/>
@@ -2190,22 +2225,22 @@
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>E03</t>
+          <t>C29</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Driver: reject an offer and accept another (needs fresh offers: reset)</t>
+          <t>Sign-in screen → "Check an existing application" for the C20 driver before documents are sent</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>The numbers in E02 move accordingly</t>
+          <t>It shows "Upload your documents", not "under review"</t>
         </is>
       </c>
       <c r="E58" s="11" t="n"/>
@@ -2214,22 +2249,22 @@
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>E04</t>
+          <t>C30</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>Merchant: Reports tab</t>
+          <t>Invitation codes still work: repeat C03 or C04 with a code from invitations.txt</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Orders, parcels and deliveries by status; matches the Admin report for that merchant</t>
+          <t>Created as before; the application is under review at once (no extra "Send for review" step)</t>
         </is>
       </c>
       <c r="E59" s="11" t="n"/>
@@ -2238,22 +2273,22 @@
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>E05</t>
+          <t>C31</t>
         </is>
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Passenger on a trip: Report a problem → Delay → write a sentence → Send</t>
+          <t>Create account → Normal user → name, email ending @example.com, password of 12+ characters → Sign up; read the code from the newest line for that email in email-codes.txt and type it</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>Confirmation; the sheet says it is not an emergency service</t>
+          <t>The code is six digits (not a long token) and finishes the sign-up; typing the same code again later does not work</t>
         </is>
       </c>
       <c r="E60" s="11" t="n"/>
@@ -2262,22 +2297,22 @@
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>E06</t>
+          <t>C32</t>
         </is>
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Send 11 reports without any being resolved</t>
+          <t>Start another email sign-up and type a wrong six-digit code five times, then the right code</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>The 11th is refused with a message about too many open reports</t>
+          <t>Each wrong code is refused; after the fifth even the right code is refused and no account exists; start again to get a new code</t>
         </is>
       </c>
       <c r="E61" s="11" t="n"/>
@@ -2286,22 +2321,22 @@
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>E07</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>Admin: Incidents</t>
+          <t>In the six-digit box try 5 digits, 7 digits, letters, or a space in the middle</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>The report from E05 is there (see A16); after you resolve it, the passenger gets two new notifications and does not see your internal note</t>
+          <t>Refused before it is checked (the Continue button stays disabled or the API answers 400)</t>
         </is>
       </c>
       <c r="E62" s="11" t="n"/>
@@ -2310,22 +2345,22 @@
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>E08</t>
+          <t>C34</t>
         </is>
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>Smaller features</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Driver: go online/offline</t>
+          <t>Sign-in screen → Forgot password → enter the email; read the code from email-codes.txt; enter email + code + a new password. Also try an email that has no account</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>The state changes once per tap and survives closing the app</t>
+          <t>The screen says the same thing for known and unknown emails and no email is produced for the unknown one; the new password signs in, the old one does not; the same code cannot be used twice</t>
         </is>
       </c>
       <c r="E63" s="11" t="n"/>
@@ -2334,22 +2369,22 @@
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>F01</t>
+          <t>C35</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Admin site: sign in as a passenger (using a passenger's email and password)</t>
+          <t>Forgot password: type a wrong six-digit code five times, then the right one</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>The reset is locked; the right code is refused; ask for a new code</t>
         </is>
       </c>
       <c r="E64" s="11" t="n"/>
@@ -2358,22 +2393,22 @@
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>F02</t>
+          <t>C36</t>
         </is>
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>A pending merchant or driver signs in on the phone</t>
+          <t>Open registration (as C19): Driver, no invitation code, new phone such as +970590005xxx; wrong then right phone code; name, password, consents</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>Refused with a clear message</t>
+          <t>Account created with no invitation; the app says "Upload your documents", not "under review" (API: onboarding status documents_required)</t>
         </is>
       </c>
       <c r="E65" s="11" t="n"/>
@@ -2382,22 +2417,22 @@
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>F03</t>
+          <t>C37</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>After the Admin rejects a driver with a reason, sign in as that driver</t>
+          <t>Press "Send for review" (API: POST /onboarding/application/submit) with no documents, then with only the licence and registration</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>Refused</t>
+          <t>Refused with 409 documents_required, listing the missing documents (3 first, then 1); nothing is submitted</t>
         </is>
       </c>
       <c r="E66" s="11" t="n"/>
@@ -2406,22 +2441,22 @@
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>F04</t>
+          <t>C38</t>
         </is>
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>As a passenger, try to open driver or merchant screens (via the menu only; no URL tricks)</t>
+          <t>Admin site: look for that driver in the approvals queue and try to approve or reject by API before it was submitted</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>Not reachable</t>
+          <t>Not in the queue; approve and reject answer 409 application_not_submitted; the driver cannot sign in</t>
         </is>
       </c>
       <c r="E67" s="11" t="n"/>
@@ -2430,22 +2465,22 @@
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>F05</t>
+          <t>C39</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>Admin downloads a driver document, then the applicant is approved: can the applicant still upload?</t>
+          <t>Add the national ID, press "Send for review" (twice)</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>No: uploading is closed once a decision is made</t>
+          <t>Accepted ("Application under review"); a second press does nothing new; the driver is now in the admin queue with three documents</t>
         </is>
       </c>
       <c r="E68" s="11" t="n"/>
@@ -2454,42 +2489,1506 @@
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>F06</t>
+          <t>D01</t>
         </is>
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>Must NOT work (safety)</t>
+          <t>Main story (passenger, merchant, driver)</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>Look through every screen for the words "push notification", "emergency", "live GPS", "payment", "earnings" used as if they work</t>
+          <t>Passenger: open the seeded request and its match</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>None claim a feature that is not built</t>
+          <t>The request and a match result are shown</t>
         </is>
       </c>
       <c r="E69" s="11" t="n"/>
       <c r="F69" s="11" t="n"/>
     </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C70" s="10" t="inlineStr">
+        <is>
+          <t>Merchant: open the seeded order</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>Five parcels and their batch are shown</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="n"/>
+      <c r="F70" s="11" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C71" s="10" t="inlineStr">
+        <is>
+          <t>Admin: open the Matching page; if there is no match yet, run matching</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>One combined passenger+parcel match exists, with a score breakdown</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="n"/>
+      <c r="F71" s="11" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C72" s="10" t="inlineStr">
+        <is>
+          <t>Driver (the selected one): open the inbox</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>The match is there; the other driver's inbox is empty</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="n"/>
+      <c r="F72" s="11" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C73" s="10" t="inlineStr">
+        <is>
+          <t>Driver: accept the match</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>Exactly one trip is created</t>
+        </is>
+      </c>
+      <c r="E73" s="11" t="n"/>
+      <c r="F73" s="11" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C74" s="10" t="inlineStr">
+        <is>
+          <t>Driver: advance pickup → picked up → in transit (and simulate points)</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>Only the next valid action is offered each time</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="n"/>
+      <c r="F74" s="11" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>Passenger and merchant: open their trip</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>Both see the same trip and the same latest location; read-only</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="n"/>
+      <c r="F75" s="11" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C76" s="10" t="inlineStr">
+        <is>
+          <t>Passenger and merchant: bell and Notifications tab</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>A "match accepted" and "trip update" entries; tapping one clears its dot; "Mark all as read" works</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="n"/>
+      <c r="F76" s="11" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>D09</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>Driver: complete the trip</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>Trip shows completed on all three phones and in the Admin</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="n"/>
+      <c r="F77" s="11" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>Main story (passenger, merchant, driver)</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>Tracking wording</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>Anywhere location appears it is described as simulated, never as live GPS</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="n"/>
+      <c r="F78" s="11" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>Driver: Earnings/performance tab</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>Completed-trip counts shown; earnings says it is not tracked (no invented amount)</t>
+        </is>
+      </c>
+      <c r="E79" s="11" t="n"/>
+      <c r="F79" s="11" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>Same tab, acceptance rate</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>Under 5 answered offers it says the rate appears after 5; after accepting/rejecting 5 offers it shows a percentage and "x of y"</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="n"/>
+      <c r="F80" s="11" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B81" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>Driver: reject an offer and accept another (needs fresh offers: reset)</t>
+        </is>
+      </c>
+      <c r="D81" s="10" t="inlineStr">
+        <is>
+          <t>The numbers in E02 move accordingly</t>
+        </is>
+      </c>
+      <c r="E81" s="11" t="n"/>
+      <c r="F81" s="11" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="9" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>Merchant: Reports tab</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>Orders, parcels and deliveries by status; matches the Admin report for that merchant</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="n"/>
+      <c r="F82" s="11" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>Passenger on a trip: Report a problem → Delay → write a sentence → Send</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
+          <t>Confirmation; the sheet says it is not an emergency service</t>
+        </is>
+      </c>
+      <c r="E83" s="11" t="n"/>
+      <c r="F83" s="11" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>Send 11 reports without any being resolved</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>The 11th is refused with a message about too many open reports</t>
+        </is>
+      </c>
+      <c r="E84" s="11" t="n"/>
+      <c r="F84" s="11" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="9" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="B85" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>Admin: Incidents</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>The report from E05 is there (see A16); after you resolve it, the passenger gets two new notifications and does not see your internal note</t>
+        </is>
+      </c>
+      <c r="E85" s="11" t="n"/>
+      <c r="F85" s="11" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>Driver: go online/offline</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>The state changes once per tap and survives closing the app</t>
+        </is>
+      </c>
+      <c r="E86" s="11" t="n"/>
+      <c r="F86" s="11" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="9" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>Passenger (route entry switched on): home → Send a parcel → pick a route and stops, size S or M, receiver name and phone, tick the forbidden-items box → Send parcel</t>
+        </is>
+      </c>
+      <c r="D87" s="10" t="inlineStr">
+        <is>
+          <t>Submit stays disabled until everything is filled and the box is ticked; the parcel then appears under My parcels as "Finding a driver"; the receiver's phone is shown masked</t>
+        </is>
+      </c>
+      <c r="E87" s="11" t="n"/>
+      <c r="F87" s="11" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>Same form: try size L, a phone that is too short, or leave the box unticked</t>
+        </is>
+      </c>
+      <c r="D88" s="10" t="inlineStr">
+        <is>
+          <t>Large is not offered; the others block Send parcel</t>
+        </is>
+      </c>
+      <c r="E88" s="11" t="n"/>
+      <c r="F88" s="11" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>Passenger: create parcels until you have 3 in flight, then a 4th</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>The 4th is refused with a message about the maximum number of parcels</t>
+        </is>
+      </c>
+      <c r="E89" s="11" t="n"/>
+      <c r="F89" s="11" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="9" t="inlineStr">
+        <is>
+          <t>E12</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>Passenger: cancel a parcel that is still "Finding a driver" (confirm the dialog)</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="inlineStr">
+        <is>
+          <t>It becomes Cancelled and the receiver details are shown as erased; once a driver has been offered or assigned the parcel there is no Cancel button</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="n"/>
+      <c r="F90" s="11" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="9" t="inlineStr">
+        <is>
+          <t>E13</t>
+        </is>
+      </c>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>Admin: Deliveries page, "Passenger parcels" section</t>
+        </is>
+      </c>
+      <c r="D91" s="10" t="inlineStr">
+        <is>
+          <t>The parcel is listed with its tracking state in English and Arabic; no receiver name, phone or note anywhere</t>
+        </is>
+      </c>
+      <c r="E91" s="11" t="n"/>
+      <c r="F91" s="11" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>Admin → create three stops and a route, publish it (API: /admin/stops, /admin/service-routes, versions, stops, publish). Needs the route switches (the local test environment turns them on)</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>The route appears in the public route catalogue (GET /routes)</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="n"/>
+      <c r="F92" s="11" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="9" t="inlineStr">
+        <is>
+          <t>E15</t>
+        </is>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>Admin → the route's "Estimated fares" tab (API: PUT /admin/service-routes/:id/fares): set seat 15.00, parcel S 7.00, M 9.00 with a reason; then try amount 0, 12.5 agorot, a 2-letter reason, a passenger account, and the same fares again</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr">
+        <is>
+          <t>Saved with your name in the history; 0, fractions and a too-short reason are refused (400), a passenger is refused (403), saving unchanged fares answers 409 fare_unchanged</t>
+        </is>
+      </c>
+      <c r="E93" s="11" t="n"/>
+      <c r="F93" s="11" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="9" t="inlineStr">
+        <is>
+          <t>E16</t>
+        </is>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>Passenger requests 2 seats on that route (API: POST /passenger/route-requests); the Admin then raises the seat fare to 20.00; the passenger repeats the same request key, then makes a new one</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr">
+        <is>
+          <t>The route list and the request show the fare as an estimate paid directly to the driver (2 x 15.00 = 30.00); after the change the first request still says 15.00 (frozen), a new request says 20.00</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="n"/>
+      <c r="F94" s="11" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>Passenger parcel (API: POST /passenger/parcels with an Idempotency-Key): size S, receiver name and phone, forbidden-items box ticked; send the same key again</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr">
+        <is>
+          <t>Created as "Finding a driver"; the receiver phone is shown masked; the second send returns the same parcel and creates no second one; a different body with the same key is refused (409)</t>
+        </is>
+      </c>
+      <c r="E95" s="11" t="n"/>
+      <c r="F95" s="11" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>Same call with size L, a 3-digit phone, the box unticked or missing, a drop-off before the pickup, a 1-letter name, or an unknown field</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="inlineStr">
+        <is>
+          <t>Each is refused with 400 (or a 4xx for the stops); nothing is created</t>
+        </is>
+      </c>
+      <c r="E96" s="11" t="n"/>
+      <c r="F96" s="11" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>Open that parcel as another passenger, a driver, a shop owner and signed out; then the Admin parcel list (GET /admin/passenger-parcels)</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="inlineStr">
+        <is>
+          <t>Others get 404, 403 or 401; the Admin list shows the parcel but no receiver name, phone or note</t>
+        </is>
+      </c>
+      <c r="E97" s="11" t="n"/>
+      <c r="F97" s="11" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>Create parcels until 3 are in flight, then a 4th</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>The 4th is refused with 409 passenger_parcel_limit_reached</t>
+        </is>
+      </c>
+      <c r="E98" s="11" t="n"/>
+      <c r="F98" s="11" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C99" s="10" t="inlineStr">
+        <is>
+          <t>Cancel a parcel that is still "Finding a driver"; cancel it again; then create a new one</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="inlineStr">
+        <is>
+          <t>Cancelled, receiver name, phone and note erased; a second cancel is refused (409); the freed slot allows a new parcel</t>
+        </is>
+      </c>
+      <c r="E99" s="11" t="n"/>
+      <c r="F99" s="11" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="9" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>As the sender open the parcel's delivery code (API: GET /parcel-orders/:id/handover, POST .../handover/regenerate)</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>The state never shows the code; "Get a new code" returns a six-digit code once; others get 404; an Admin cannot re-issue it (403)</t>
+        </is>
+      </c>
+      <c r="E100" s="11" t="n"/>
+      <c r="F100" s="11" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>Shop owner → bulk orders (API: POST /merchant/orders/bulk/preview): paste a CSV with 5 rows (one has size Q); also try as a passenger</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="inlineStr">
+        <is>
+          <t>The preview lists the valid orders, the bad row with its row number and an Arabic message, and a batch plan; nothing is created; passengers are refused</t>
+        </is>
+      </c>
+      <c r="E101" s="11" t="n"/>
+      <c r="F101" s="11" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="9" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>Submit the CSV without an Idempotency-Key, then with the bad row and without "skip invalid"</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>Both are refused (400) and no order is created</t>
+        </is>
+      </c>
+      <c r="E102" s="11" t="n"/>
+      <c r="F102" s="11" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>Submit the valid rows with an Idempotency-Key, then send exactly the same upload again; then submit with "skip invalid"</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>First: 3 orders created; the retry creates nothing (all "replayed", the same order numbers, the order list still has 3); skipping the bad row creates the valid ones and reports 1 failed</t>
+        </is>
+      </c>
+      <c r="E103" s="11" t="n"/>
+      <c r="F103" s="11" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>Preview or submit a CSV with 51 rows; then one with exactly 50</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>51 rows: rejected as a whole with csv_too_many_rows and nothing created; 50 rows are accepted by the preview</t>
+        </is>
+      </c>
+      <c r="E104" s="11" t="n"/>
+      <c r="F104" s="11" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="9" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>Passenger assistant with no AI key (Assistant on the passenger home): "from Bab Al-Zawiya to Bethlehem Center tomorrow at 8am with 2 seats", and the same in Arabic</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr">
+        <is>
+          <t>The rule-based fallback fills pickup, destination, time and 2 seats for review; admins and signed-out users cannot use it; an empty message is refused</t>
+        </is>
+      </c>
+      <c r="E105" s="11" t="n"/>
+      <c r="F105" s="11" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="9" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>Ask the assistant for a ride to Nablus (English and Arabic)</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>A clear reply that the place is not supported yet, listing the supported places as suggestions</t>
+        </is>
+      </c>
+      <c r="E106" s="11" t="n"/>
+      <c r="F106" s="11" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>Send the assistant something it cannot read; then Admin → Incidents → uncertain assistant requests (API: GET /admin/ai-uncertain-requests); resolve it with a note</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="inlineStr">
+        <is>
+          <t>A clear request is not queued; the unclear one is queued once with its reason and no passenger identity; resolving needs the current revision, a resolved one cannot be resolved again, and the open count drops</t>
+        </is>
+      </c>
+      <c r="E107" s="11" t="n"/>
+      <c r="F107" s="11" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>E30</t>
+        </is>
+      </c>
+      <c r="B108" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>Passenger with an accepted trip: step the simulated driver (Simulate step) until it is near the pickup, then open Notifications</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="inlineStr">
+        <is>
+          <t>Exactly one "your driver is approaching" notification (no coordinates in it), however many steps follow; the shop owner gets none</t>
+        </is>
+      </c>
+      <c r="E108" s="11" t="n"/>
+      <c r="F108" s="11" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t>E31</t>
+        </is>
+      </c>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>Driver on an in-transit parcel trip: try Delivered with the normal status button, then confirm with no code, and try to confirm as the passenger or shop owner</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>The status route refuses (409 delivery_confirmation_required), no code is 400, other roles 403; the trip stays in transit</t>
+        </is>
+      </c>
+      <c r="E109" s="11" t="n"/>
+      <c r="F109" s="11" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>E32</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>Shop owner: Get a new code for the order (API: POST /parcel-orders/:id/handover/regenerate); the driver tries to read or re-issue it</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>A six-digit code is returned once, attempts remaining 5; the driver gets 404 for both</t>
+        </is>
+      </c>
+      <c r="E110" s="11" t="n"/>
+      <c r="F110" s="11" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="9" t="inlineStr">
+        <is>
+          <t>E33</t>
+        </is>
+      </c>
+      <c r="B111" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>Driver enters a wrong code five times, then the right code; then the shop owner gets a new code</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>Wrong codes are refused (422); after five, even the right code is refused (429 handover_locked) and the order shows locked; a new code unlocks it</t>
+        </is>
+      </c>
+      <c r="E111" s="11" t="n"/>
+      <c r="F111" s="11" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="inlineStr">
+        <is>
+          <t>E34</t>
+        </is>
+      </c>
+      <c r="B112" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>Driver enters the right code; the Admin opens the trip (API: GET /admin/trips/:id)</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>The trip becomes delivered; the Admin sees it confirmed by receiver code and not flagged; the code is shown nowhere; confirming again is refused</t>
+        </is>
+      </c>
+      <c r="E112" s="11" t="n"/>
+      <c r="F112" s="11" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="9" t="inlineStr">
+        <is>
+          <t>E35</t>
+        </is>
+      </c>
+      <c r="B113" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>Passenger rates the finished trip: before completion, 0 and 6 stars, then 5 stars, then again; drivers and shop owners try to rate or read it</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>Before completion 409 trip_not_completed; 0, 6 and 4.5 are 400; 5 stars saved (201); a second rating 409 trip_already_rated; the passenger can see only their own rating; drivers get 403/404 and no driver screen or API shows a star rating</t>
+        </is>
+      </c>
+      <c r="E113" s="11" t="n"/>
+      <c r="F113" s="11" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="9" t="inlineStr">
+        <is>
+          <t>E36</t>
+        </is>
+      </c>
+      <c r="B114" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>After the trip: driver trust score (Admin → user detail) and npm run trust:recompute -w @masari/api against the demo database</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>A whole number from 0 to 100 with its breakdown and calculation time; the Admin sees the same number; the job reports 0 failed and gives the same score when run again</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="n"/>
+      <c r="F114" s="11" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="inlineStr">
+        <is>
+          <t>E37</t>
+        </is>
+      </c>
+      <c r="B115" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>Second trip: the driver chooses "Receiver unavailable" with no reason, a 9-character reason, a 301-character reason, then a proper reason</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>The first three are refused (400); the proper one delivers the trip, the Admin trip list and detail show it flagged with the reason, and the sender sees how it was confirmed</t>
+        </is>
+      </c>
+      <c r="E115" s="11" t="n"/>
+      <c r="F115" s="11" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="9" t="inlineStr">
+        <is>
+          <t>E38</t>
+        </is>
+      </c>
+      <c r="B116" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>Admin approves a new driver with document dates (API: expiry on approve): try a licence date in the past, then valid dates</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>A past date is refused (400 expiry_date_in_past); valid dates are saved and the driver appears under "Expiring soon" (within 30 days); a driver cannot read that list</t>
+        </is>
+      </c>
+      <c r="E116" s="11" t="n"/>
+      <c r="F116" s="11" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="9" t="inlineStr">
+        <is>
+          <t>E39</t>
+        </is>
+      </c>
+      <c r="B117" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>Run the expiry job (npm run documents:expiry -w @masari/api) with the licence ending in 5 days, twice</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>The driver gets one "document expires soon" reminder; the second run adds none; the driver is still approved</t>
+        </is>
+      </c>
+      <c r="E117" s="11" t="n"/>
+      <c r="F117" s="11" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="9" t="inlineStr">
+        <is>
+          <t>E40</t>
+        </is>
+      </c>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>Set the licence date to yesterday (database edit on masari_demo) and run the job again; then try to go online</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>The driver becomes "documents expired", is unverified, gets a notification, and going online is refused with 403 driver_documents_expired; a second run restricts nobody twice; the driver still signs in; the Admin sees the driver under "Awaiting driver"</t>
+        </is>
+      </c>
+      <c r="E118" s="11" t="n"/>
+      <c r="F118" s="11" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="9" t="inlineStr">
+        <is>
+          <t>E41</t>
+        </is>
+      </c>
+      <c r="B119" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>Driver renewal (API: /driver/document-renewal): submit with no file, upload a text file, upload a photo, submit</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>No file: 409; text file: 415; with a photo the application goes to the Admin re-review queue; going online is still refused; passengers cannot use the renewal area</t>
+        </is>
+      </c>
+      <c r="E119" s="11" t="n"/>
+      <c r="F119" s="11" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="9" t="inlineStr">
+        <is>
+          <t>E42</t>
+        </is>
+      </c>
+      <c r="B120" s="10" t="inlineStr">
+        <is>
+          <t>Smaller features</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>Admin approves the renewal: first without new dates, then with a new licence date</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>Without new dates it is refused (400); with a new date the driver is approved and verified again at once, the history shows expired and renewal submitted, going online is no longer refused for documents, and the job does not restrict them again</t>
+        </is>
+      </c>
+      <c r="E120" s="11" t="n"/>
+      <c r="F120" s="11" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="9" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B121" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>Admin site: sign in as a passenger (using a passenger's email and password)</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>Refused</t>
+        </is>
+      </c>
+      <c r="E121" s="11" t="n"/>
+      <c r="F121" s="11" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
+      <c r="B122" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>A pending merchant or driver signs in on the phone</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>Refused with a clear message</t>
+        </is>
+      </c>
+      <c r="E122" s="11" t="n"/>
+      <c r="F122" s="11" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="inlineStr">
+        <is>
+          <t>F03</t>
+        </is>
+      </c>
+      <c r="B123" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>After the Admin rejects a driver with a reason, sign in as that driver</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>Refused</t>
+        </is>
+      </c>
+      <c r="E123" s="11" t="n"/>
+      <c r="F123" s="11" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="9" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>As a passenger, try to open driver or merchant screens (via the menu only; no URL tricks)</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>Not reachable</t>
+        </is>
+      </c>
+      <c r="E124" s="11" t="n"/>
+      <c r="F124" s="11" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="B125" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>Admin downloads a driver document, then the applicant is approved: can the applicant still upload?</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>No: uploading is closed once a decision is made</t>
+        </is>
+      </c>
+      <c r="E125" s="11" t="n"/>
+      <c r="F125" s="11" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>Look through every screen for the words "push notification", "emergency", "live GPS", "payment", "earnings" used as if they work</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>None claim a feature that is not built</t>
+        </is>
+      </c>
+      <c r="E126" s="11" t="n"/>
+      <c r="F126" s="11" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>F07</t>
+        </is>
+      </c>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>With the open-registration switch off (OPEN_DRIVER_MERCHANT_SIGNUP_ENABLED=false, the default everywhere except the local test environment), choose Driver and leave the invitation code empty</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>The code field is required; sending without one is refused and no code is produced</t>
+        </is>
+      </c>
+      <c r="E127" s="11" t="n"/>
+      <c r="F127" s="11" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="9" t="inlineStr">
+        <is>
+          <t>F08</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Call POST /api/v1/onboarding/application/submit with a pending driver or shop owner session that is missing a required document (any HTTP client)</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="inlineStr">
+        <is>
+          <t>409 documents_required, listing what is missing; the application is not submitted</t>
+        </is>
+      </c>
+      <c r="E128" s="11" t="n"/>
+      <c r="F128" s="11" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="9" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="B129" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>Passenger role without an invitation code, even with the switch on</t>
+        </is>
+      </c>
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>Refused; passengers always register by email or Google</t>
+        </is>
+      </c>
+      <c r="E129" s="11" t="n"/>
+      <c r="F129" s="11" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="9" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>Must NOT work (safety)</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>A submitted driver deletes the only file of a required kind</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="inlineStr">
+        <is>
+          <t>Refused (documents_required); replacing it by adding a second file first works</t>
+        </is>
+      </c>
+      <c r="E130" s="11" t="n"/>
+      <c r="F130" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F69"/>
-  <conditionalFormatting sqref="E2:E69">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+  <autoFilter ref="A1:F130"/>
+  <conditionalFormatting sqref="E2:E130">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"PASS"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
       <formula>"FAIL"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
       <formula>"SKIP"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E69" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Pick from the list" error="Choose PASS, FAIL or SKIP." type="list">
+    <dataValidation sqref="E2:E130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,SKIP"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2553,19 +4052,19 @@
         </is>
       </c>
       <c r="B2" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$69,"A*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$130,"A*")</f>
         <v/>
       </c>
       <c r="C2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"A*",Tests!$E$2:$E$69,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"A*",Tests!$E$2:$E$130,"PASS")</f>
         <v/>
       </c>
       <c r="D2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"A*",Tests!$E$2:$E$69,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"A*",Tests!$E$2:$E$130,"FAIL")</f>
         <v/>
       </c>
       <c r="E2" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"A*",Tests!$E$2:$E$69,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"A*",Tests!$E$2:$E$130,"SKIP")</f>
         <v/>
       </c>
       <c r="F2" s="13">
@@ -2580,19 +4079,19 @@
         </is>
       </c>
       <c r="B3" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$69,"B*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$130,"B*")</f>
         <v/>
       </c>
       <c r="C3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"B*",Tests!$E$2:$E$69,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"B*",Tests!$E$2:$E$130,"PASS")</f>
         <v/>
       </c>
       <c r="D3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"B*",Tests!$E$2:$E$69,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"B*",Tests!$E$2:$E$130,"FAIL")</f>
         <v/>
       </c>
       <c r="E3" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"B*",Tests!$E$2:$E$69,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"B*",Tests!$E$2:$E$130,"SKIP")</f>
         <v/>
       </c>
       <c r="F3" s="13">
@@ -2603,23 +4102,23 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Phone: sign-up with invitation</t>
+          <t>Phone: sign-up (invitation or open)</t>
         </is>
       </c>
       <c r="B4" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$69,"C*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$130,"C*")</f>
         <v/>
       </c>
       <c r="C4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"C*",Tests!$E$2:$E$69,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"C*",Tests!$E$2:$E$130,"PASS")</f>
         <v/>
       </c>
       <c r="D4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"C*",Tests!$E$2:$E$69,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"C*",Tests!$E$2:$E$130,"FAIL")</f>
         <v/>
       </c>
       <c r="E4" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"C*",Tests!$E$2:$E$69,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"C*",Tests!$E$2:$E$130,"SKIP")</f>
         <v/>
       </c>
       <c r="F4" s="13">
@@ -2634,19 +4133,19 @@
         </is>
       </c>
       <c r="B5" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$69,"D*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$130,"D*")</f>
         <v/>
       </c>
       <c r="C5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"D*",Tests!$E$2:$E$69,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"D*",Tests!$E$2:$E$130,"PASS")</f>
         <v/>
       </c>
       <c r="D5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"D*",Tests!$E$2:$E$69,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"D*",Tests!$E$2:$E$130,"FAIL")</f>
         <v/>
       </c>
       <c r="E5" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"D*",Tests!$E$2:$E$69,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"D*",Tests!$E$2:$E$130,"SKIP")</f>
         <v/>
       </c>
       <c r="F5" s="13">
@@ -2661,19 +4160,19 @@
         </is>
       </c>
       <c r="B6" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$69,"E*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$130,"E*")</f>
         <v/>
       </c>
       <c r="C6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"E*",Tests!$E$2:$E$69,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"E*",Tests!$E$2:$E$130,"PASS")</f>
         <v/>
       </c>
       <c r="D6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"E*",Tests!$E$2:$E$69,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"E*",Tests!$E$2:$E$130,"FAIL")</f>
         <v/>
       </c>
       <c r="E6" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"E*",Tests!$E$2:$E$69,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"E*",Tests!$E$2:$E$130,"SKIP")</f>
         <v/>
       </c>
       <c r="F6" s="13">
@@ -2688,19 +4187,19 @@
         </is>
       </c>
       <c r="B7" s="13">
-        <f>COUNTIF(Tests!$A$2:$A$69,"F*")</f>
+        <f>COUNTIF(Tests!$A$2:$A$130,"F*")</f>
         <v/>
       </c>
       <c r="C7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"F*",Tests!$E$2:$E$69,"PASS")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"F*",Tests!$E$2:$E$130,"PASS")</f>
         <v/>
       </c>
       <c r="D7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"F*",Tests!$E$2:$E$69,"FAIL")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"F*",Tests!$E$2:$E$130,"FAIL")</f>
         <v/>
       </c>
       <c r="E7" s="13">
-        <f>COUNTIFS(Tests!$A$2:$A$69,"F*",Tests!$E$2:$E$69,"SKIP")</f>
+        <f>COUNTIFS(Tests!$A$2:$A$130,"F*",Tests!$E$2:$E$130,"SKIP")</f>
         <v/>
       </c>
       <c r="F7" s="13">
@@ -2736,7 +4235,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>The counts update by themselves as you fill in the Tests sheet.</t>
         </is>

</xml_diff>